<commit_message>
actualización master y diccionario
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/oscarj_iadb_org/Documents/Desktop/work/github repositories/historia-fiscal-y-monetaria-Ecuador/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EDU\repositorios\historia-fiscal-y-monetaria-Ecuador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4C63F6194B02D715F12B5BCB046EF0A713351A4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBF8217C-8137-4933-9794-891101B26DD7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF71427-B386-4D30-9003-A14FF24E23E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20385" yWindow="1200" windowWidth="22950" windowHeight="16905" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19920" yWindow="2310" windowWidth="27330" windowHeight="17385" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadatos" sheetId="1" r:id="rId1"/>
@@ -461,7 +461,7 @@
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
     <col min="2" max="2" width="48.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1204,7 +1204,7 @@
         <v>393.63886258319837</v>
       </c>
       <c r="T25">
-        <f t="shared" ref="T25:T56" si="1">S25/F25*$F$89</f>
+        <f>S25/F25*$F$89</f>
         <v>4276604.8351706136</v>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
         <v>432.30741138996598</v>
       </c>
       <c r="T26">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="T25:T56" si="1">S26/F26*$F$89</f>
         <v>4200688.6932424754</v>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
         <v>101726</v>
       </c>
       <c r="T89">
-        <f t="shared" ref="T89:T120" si="5">S89/F89*$F$89</f>
+        <f t="shared" ref="T89:T98" si="5">S89/F89*$F$89</f>
         <v>101726</v>
       </c>
       <c r="U89">
@@ -4711,7 +4711,7 @@
         <v>3.5546017070164598E-3</v>
       </c>
       <c r="E16">
-        <f t="shared" ref="E15:E43" si="0">B16*$D$102</f>
+        <f t="shared" ref="E16:E43" si="0">B16*$D$102</f>
         <v>2.5808578027034261E-3</v>
       </c>
     </row>

</xml_diff>